<commit_message>
BinhLH_Remove payout percentage from dashboard header
Update admin dashboard template to change the column label from "Payout (90%)" to a generic "Payout". Also update test spreadsheet files (booking_test_data.xlsx, booking_test_report.xlsx, wishlist_test_report.xlsx). This removes the hardcoded 90% label so the UI no longer implies a fixed payout percentage.
</commit_message>
<xml_diff>
--- a/booking_test_report.xlsx
+++ b/booking_test_report.xlsx
@@ -44,10 +44,10 @@
     <t>customer_binh</t>
   </si>
   <si>
-    <t>Thảo Điểm</t>
-  </si>
-  <si>
-    <t>Deluxe Room</t>
+    <t>Vinpearl Resort Nha Trang</t>
+  </si>
+  <si>
+    <t>Deluxe Sea View</t>
   </si>
   <si>
     <t>Đăng nhập -&gt; Xem phòng -&gt; Đặt phòng Deluxe -&gt; Điền thông tin -&gt; Đặt phòng -&gt; Bypass thanh toán -&gt; Kiểm tra trạng thái Confirmed tại Lịch sử</t>
@@ -56,7 +56,7 @@
     <t>PASS</t>
   </si>
   <si>
-    <t>38281</t>
+    <t>13361</t>
   </si>
   <si>
     <t>Happy Path PASS: Booking created and bypass payment confirmed status successfully.</t>
@@ -68,7 +68,7 @@
     <t>Không đăng nhập -&gt; Truy cập trực tiếp trang Checkout -&gt; Xác nhận bị chặn và chuyển hướng về trang Đăng nhập</t>
   </si>
   <si>
-    <t>1931</t>
+    <t>1776</t>
   </si>
   <si>
     <t>Security Path PASS: Unauthenticated user successfully redirected to login page.</t>
@@ -80,7 +80,7 @@
     <t>Đăng nhập -&gt; Vào Checkout -&gt; Bỏ trống Họ tên bắt buộc -&gt; Bấm đặt phòng -&gt; Xác nhận trình duyệt chặn submit (URL giữ nguyên ở /booking)</t>
   </si>
   <si>
-    <t>6131</t>
+    <t>21543</t>
   </si>
   <si>
     <t>Validation Path PASS: Form submission prevented due to missing required info.</t>
@@ -89,13 +89,13 @@
     <t>TC_BK_04</t>
   </si>
   <si>
-    <t>owner_thaodiem</t>
+    <t>owner_vinpearl</t>
   </si>
   <si>
     <t>Đăng nhập bằng tài khoản Chủ khách sạn (Owner) -&gt; Truy cập trang Checkout -&gt; Xác nhận bị chặn và chuyển hướng về trang Home</t>
   </si>
   <si>
-    <t>2396</t>
+    <t>3102</t>
   </si>
   <si>
     <t>Role Validation Path PASS: Owner redirected to Home page.</t>
@@ -107,7 +107,7 @@
     <t>Đăng nhập -&gt; Truy cập Checkout với ID khách sạn không tồn tại (9999) -&gt; Xác nhận bị chặn và chuyển hướng về trang Khách sạn</t>
   </si>
   <si>
-    <t>2811</t>
+    <t>2520</t>
   </si>
   <si>
     <t>Business Rule Path PASS: Non-existent/Inactive hotel booking redirected to hotels page.</t>
@@ -192,9 +192,9 @@
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="10.84765625" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="14.80078125" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="10.734375" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="11.625" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="13.5546875" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="22.01171875" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="14.140625" customWidth="true" bestFit="true"/>
     <col min="5" max="5" width="114.921875" customWidth="true" bestFit="true"/>
     <col min="6" max="6" width="6.06640625" customWidth="true" bestFit="true"/>
     <col min="7" max="7" width="17.5546875" customWidth="true" bestFit="true"/>

</xml_diff>

<commit_message>
BinhLH_Refactor review to feedback across the codebase
- Renamed folders HomePage to homepage and User to user.
- Refactored terminology from review to feedback.
- Updated Java entities, HTML templates, CSS, JS and database SQL schemas.
- Modified Entity database mappings (Table, Column, JoinColumn) and Database scripts.
- Renamed Java classes and controllers related to Feedback.
</commit_message>
<xml_diff>
--- a/booking_test_report.xlsx
+++ b/booking_test_report.xlsx
@@ -56,7 +56,7 @@
     <t>PASS</t>
   </si>
   <si>
-    <t>13361</t>
+    <t>15199</t>
   </si>
   <si>
     <t>Happy Path PASS: Booking created and bypass payment confirmed status successfully.</t>
@@ -68,7 +68,7 @@
     <t>Không đăng nhập -&gt; Truy cập trực tiếp trang Checkout -&gt; Xác nhận bị chặn và chuyển hướng về trang Đăng nhập</t>
   </si>
   <si>
-    <t>1776</t>
+    <t>2306</t>
   </si>
   <si>
     <t>Security Path PASS: Unauthenticated user successfully redirected to login page.</t>
@@ -80,7 +80,7 @@
     <t>Đăng nhập -&gt; Vào Checkout -&gt; Bỏ trống Họ tên bắt buộc -&gt; Bấm đặt phòng -&gt; Xác nhận trình duyệt chặn submit (URL giữ nguyên ở /booking)</t>
   </si>
   <si>
-    <t>21543</t>
+    <t>7624</t>
   </si>
   <si>
     <t>Validation Path PASS: Form submission prevented due to missing required info.</t>
@@ -95,7 +95,7 @@
     <t>Đăng nhập bằng tài khoản Chủ khách sạn (Owner) -&gt; Truy cập trang Checkout -&gt; Xác nhận bị chặn và chuyển hướng về trang Home</t>
   </si>
   <si>
-    <t>3102</t>
+    <t>3074</t>
   </si>
   <si>
     <t>Role Validation Path PASS: Owner redirected to Home page.</t>
@@ -107,7 +107,7 @@
     <t>Đăng nhập -&gt; Truy cập Checkout với ID khách sạn không tồn tại (9999) -&gt; Xác nhận bị chặn và chuyển hướng về trang Khách sạn</t>
   </si>
   <si>
-    <t>2520</t>
+    <t>3426</t>
   </si>
   <si>
     <t>Business Rule Path PASS: Non-existent/Inactive hotel booking redirected to hotels page.</t>

</xml_diff>

<commit_message>
BinhLH_Update dashboard date range picker and remove customer gender column
- Update admin dashboard date filter to use Flatpickr pill-style form matching the home page

- Remove gender column and check constraint from customers table in database schema and sample data insertion scripts

- Remove gender attribute and getter/setter from Customer Java Entity class

- Update hotel_booking.dbml file accordingly
</commit_message>
<xml_diff>
--- a/booking_test_report.xlsx
+++ b/booking_test_report.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="34">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -53,22 +53,31 @@
     <t>Đăng nhập -&gt; Xem phòng -&gt; Đặt phòng Deluxe -&gt; Điền thông tin -&gt; Đặt phòng -&gt; Bypass thanh toán -&gt; Kiểm tra trạng thái Confirmed tại Lịch sử</t>
   </si>
   <si>
+    <t>FAIL</t>
+  </si>
+  <si>
+    <t>79767</t>
+  </si>
+  <si>
+    <t>Error: Expected condition failed: waiting for element found by By.xpath: //div[contains(@class, 'room-card') and .//div[contains(@class, 'room-type-title') and contains(text(), 'Deluxe Sea View')]]/descendant::a[contains(text(), 'Booking') or contains(@id, 'booking-btn')] to be clickable, but the element was not found: org.openqa.selenium.NoSuchElementException: no such element: Unable to locate element: {"method":"xpath","selector":"//div[contains(@class, 'room-card') and .//div[contains(@class, 'room-type-title') and contains(text(), 'Deluxe Sea View')]]/descendant::a[contains(text(), 'Booking') or contains(@id, 'booking-btn')]"}.
+(tried for 12 seconds with 500 milliseconds interval)
+Build info: version: '4.43.0', revision: 'dd0f534'
+System info: os.name: 'Windows 11', os.arch: 'amd64', os.version: '10.0', java.version: '25.0.2'
+Driver info: org.openqa.selenium.chrome.ChromeDriver
+Capabilities {acceptInsecureCerts: false, browserName: chrome, browserVersion: 150.0.7871.102, chrome: {chromedriverVersion: 150.0.7871.115 (25f5b661e5b..., userDataDir: C:\Users\luuhu\AppData\Loca...}, fedcm:accounts: true, goog:chromeOptions: {debuggerAddress: localhost:50388}, goog:processID: 25344, networkConnectionEnabled: false, pageLoadStrategy: normal, platformName: windows, proxy: Proxy(), se:cdp: ws://localhost:50388/devtoo..., se:cdpVersion: 150.0.7871.102, setWindowRect: true, strictFileInteractability: false, timeouts: {implicit: 0, pageLoad: 300000, script: 30000}, unhandledPromptBehavior: dismiss and notify, webauthn:extension:credBlob: true, webauthn:extension:largeBlob: true, webauthn:extension:minPinLength: true, webauthn:extension:prf: true, webauthn:virtualAuthenticators: true}
+Session ID: 4eb091362da0a83a841897916baa6f85</t>
+  </si>
+  <si>
+    <t>TC_BK_02</t>
+  </si>
+  <si>
+    <t>Không đăng nhập -&gt; Truy cập trực tiếp trang Checkout -&gt; Xác nhận bị chặn và chuyển hướng về trang Đăng nhập</t>
+  </si>
+  <si>
     <t>PASS</t>
   </si>
   <si>
-    <t>15199</t>
-  </si>
-  <si>
-    <t>Happy Path PASS: Booking created and bypass payment confirmed status successfully.</t>
-  </si>
-  <si>
-    <t>TC_BK_02</t>
-  </si>
-  <si>
-    <t>Không đăng nhập -&gt; Truy cập trực tiếp trang Checkout -&gt; Xác nhận bị chặn và chuyển hướng về trang Đăng nhập</t>
-  </si>
-  <si>
-    <t>2306</t>
+    <t>2438</t>
   </si>
   <si>
     <t>Security Path PASS: Unauthenticated user successfully redirected to login page.</t>
@@ -80,7 +89,7 @@
     <t>Đăng nhập -&gt; Vào Checkout -&gt; Bỏ trống Họ tên bắt buộc -&gt; Bấm đặt phòng -&gt; Xác nhận trình duyệt chặn submit (URL giữ nguyên ở /booking)</t>
   </si>
   <si>
-    <t>7624</t>
+    <t>7367</t>
   </si>
   <si>
     <t>Validation Path PASS: Form submission prevented due to missing required info.</t>
@@ -95,7 +104,7 @@
     <t>Đăng nhập bằng tài khoản Chủ khách sạn (Owner) -&gt; Truy cập trang Checkout -&gt; Xác nhận bị chặn và chuyển hướng về trang Home</t>
   </si>
   <si>
-    <t>3074</t>
+    <t>3259</t>
   </si>
   <si>
     <t>Role Validation Path PASS: Owner redirected to Home page.</t>
@@ -107,7 +116,7 @@
     <t>Đăng nhập -&gt; Truy cập Checkout với ID khách sạn không tồn tại (9999) -&gt; Xác nhận bị chặn và chuyển hướng về trang Khách sạn</t>
   </si>
   <si>
-    <t>3426</t>
+    <t>3281</t>
   </si>
   <si>
     <t>Business Rule Path PASS: Non-existent/Inactive hotel booking redirected to hotels page.</t>
@@ -198,7 +207,7 @@
     <col min="5" max="5" width="114.921875" customWidth="true" bestFit="true"/>
     <col min="6" max="6" width="6.06640625" customWidth="true" bestFit="true"/>
     <col min="7" max="7" width="17.5546875" customWidth="true" bestFit="true"/>
-    <col min="8" max="8" width="71.39453125" customWidth="true" bestFit="true"/>
+    <col min="8" max="8" width="255.0" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -243,7 +252,7 @@
       <c r="E2" t="s" s="0">
         <v>12</v>
       </c>
-      <c r="F2" t="s" s="2">
+      <c r="F2" t="s" s="3">
         <v>13</v>
       </c>
       <c r="G2" t="s" s="0">
@@ -270,18 +279,18 @@
         <v>17</v>
       </c>
       <c r="F3" t="s" s="2">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="G3" t="s" s="0">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H3" t="s" s="0">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B4" t="s" s="0">
         <v>9</v>
@@ -293,24 +302,24 @@
         <v>11</v>
       </c>
       <c r="E4" t="s" s="0">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F4" t="s" s="2">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="G4" t="s" s="0">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="H4" t="s" s="0">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C5" t="s" s="0">
         <v>10</v>
@@ -319,21 +328,21 @@
         <v>11</v>
       </c>
       <c r="E5" t="s" s="0">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F5" t="s" s="2">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="G5" t="s" s="0">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="H5" t="s" s="0">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B6" t="s" s="0">
         <v>9</v>
@@ -345,16 +354,16 @@
         <v>11</v>
       </c>
       <c r="E6" t="s" s="0">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F6" t="s" s="2">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="G6" t="s" s="0">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H6" t="s" s="0">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
BinhLH_Add otpAttempts field to User entity and update related OTP templates and controllers
Detailed changes: Add otpAttempts field with default 0 in User.java along with getter/setter. Update ProfileController, AdminDashboardController, and OTP verification HTML templates to support enhanced OTP tracking and user profile verification flows.
</commit_message>
<xml_diff>
--- a/booking_test_report.xlsx
+++ b/booking_test_report.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="34">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -53,22 +53,33 @@
     <t>Đăng nhập -&gt; Xem phòng -&gt; Đặt phòng Deluxe -&gt; Điền thông tin -&gt; Đặt phòng -&gt; Bypass thanh toán -&gt; Kiểm tra trạng thái Confirmed tại Lịch sử</t>
   </si>
   <si>
+    <t>FAIL</t>
+  </si>
+  <si>
+    <t>263444</t>
+  </si>
+  <si>
+    <t>Error: invalid session id: session deleted as the browser has closed the connection
+from disconnected: unable to send message to renderer
+  (Session info: chrome=150.0.7871.129)
+Build info: version: '4.31.0', revision: '1ef9f18787*'
+System info: os.name: 'Windows 11', os.arch: 'amd64', os.version: '10.0', java.version: '25.0.2'
+Driver info: org.openqa.selenium.chrome.ChromeDriver
+Command: [dafd9034528d502f159848ef142c9a87, findElement {using=id, value=payment-data}]
+Capabilities {acceptInsecureCerts: false, browserName: chrome, browserVersion: 150.0.7871.129, chrome: {chromedriverVersion: 150.0.7871.124 (9261fd0a595..., userDataDir: C:\Users\luuhu\AppData\Loca...}, fedcm:accounts: true, goog:chromeOptions: {debuggerAddress: localhost:58202}, goog:processID: 16492, networkConnectionEnabled: false, pageLoadStrategy: normal, platformName: windows, proxy: Proxy(), se:cdp: ws://localhost:58202/devtoo..., se:cdpVersion: 150.0.7871.129, setWindowRect: true, strictFileInteractability: false, timeouts: {implicit: 0, pageLoad: 300000, script: 30000}, unhandledPromptBehavior: dismiss and notify, webauthn:extension:credBlob: true, webauthn:extension:largeBlob: true, webauthn:extension:minPinLength: true, webauthn:extension:prf: true, webauthn:virtualAuthenticators: true}
+Session ID: dafd9034528d502f159848ef142c9a87</t>
+  </si>
+  <si>
+    <t>TC_BK_02</t>
+  </si>
+  <si>
+    <t>Không đăng nhập -&gt; Truy cập trực tiếp trang Checkout -&gt; Xác nhận bị chặn và chuyển hướng về trang Đăng nhập</t>
+  </si>
+  <si>
     <t>PASS</t>
   </si>
   <si>
-    <t>7998</t>
-  </si>
-  <si>
-    <t>Happy Path PASS: Booking created and bypass payment confirmed status successfully.</t>
-  </si>
-  <si>
-    <t>TC_BK_02</t>
-  </si>
-  <si>
-    <t>Không đăng nhập -&gt; Truy cập trực tiếp trang Checkout -&gt; Xác nhận bị chặn và chuyển hướng về trang Đăng nhập</t>
-  </si>
-  <si>
-    <t>1238</t>
+    <t>1509</t>
   </si>
   <si>
     <t>Security Path PASS: Unauthenticated user successfully redirected to login page.</t>
@@ -80,7 +91,7 @@
     <t>Đăng nhập -&gt; Vào Checkout -&gt; Bỏ trống Họ tên bắt buộc -&gt; Bấm đặt phòng -&gt; Xác nhận trình duyệt chặn submit (URL giữ nguyên ở /booking)</t>
   </si>
   <si>
-    <t>6397</t>
+    <t>6636</t>
   </si>
   <si>
     <t>Validation Path PASS: Form submission prevented due to missing required info.</t>
@@ -95,7 +106,7 @@
     <t>Đăng nhập bằng tài khoản Chủ khách sạn (Owner) -&gt; Truy cập trang Checkout -&gt; Xác nhận bị chặn và chuyển hướng về trang Home</t>
   </si>
   <si>
-    <t>2666</t>
+    <t>2541</t>
   </si>
   <si>
     <t>Role Validation Path PASS: Owner redirected to Home page.</t>
@@ -107,7 +118,7 @@
     <t>Đăng nhập -&gt; Truy cập Checkout với ID khách sạn không tồn tại (9999) -&gt; Xác nhận bị chặn và chuyển hướng về trang Khách sạn</t>
   </si>
   <si>
-    <t>2494</t>
+    <t>2145</t>
   </si>
   <si>
     <t>Business Rule Path PASS: Non-existent/Inactive hotel booking redirected to hotels page.</t>
@@ -198,7 +209,7 @@
     <col min="5" max="5" width="114.921875" customWidth="true" bestFit="true"/>
     <col min="6" max="6" width="6.06640625" customWidth="true" bestFit="true"/>
     <col min="7" max="7" width="17.5546875" customWidth="true" bestFit="true"/>
-    <col min="8" max="8" width="71.39453125" customWidth="true" bestFit="true"/>
+    <col min="8" max="8" width="255.0" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -243,7 +254,7 @@
       <c r="E2" t="s" s="0">
         <v>12</v>
       </c>
-      <c r="F2" t="s" s="2">
+      <c r="F2" t="s" s="3">
         <v>13</v>
       </c>
       <c r="G2" t="s" s="0">
@@ -270,18 +281,18 @@
         <v>17</v>
       </c>
       <c r="F3" t="s" s="2">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="G3" t="s" s="0">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H3" t="s" s="0">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B4" t="s" s="0">
         <v>9</v>
@@ -293,24 +304,24 @@
         <v>11</v>
       </c>
       <c r="E4" t="s" s="0">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F4" t="s" s="2">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="G4" t="s" s="0">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="H4" t="s" s="0">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C5" t="s" s="0">
         <v>10</v>
@@ -319,21 +330,21 @@
         <v>11</v>
       </c>
       <c r="E5" t="s" s="0">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F5" t="s" s="2">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="G5" t="s" s="0">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="H5" t="s" s="0">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B6" t="s" s="0">
         <v>9</v>
@@ -345,16 +356,16 @@
         <v>11</v>
       </c>
       <c r="E6" t="s" s="0">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F6" t="s" s="2">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="G6" t="s" s="0">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H6" t="s" s="0">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>